<commit_message>
Update performance and report files; add new Jupyter notebook for Lesson 3 project
</commit_message>
<xml_diff>
--- a/Lesson 2 project/report.xlsx
+++ b/Lesson 2 project/report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AAIS\Lesson 2 project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A0437CF-2C07-4ED9-B8CA-1040AE49828F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC02DDC4-F465-4EF9-B368-1AD226D83C55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="41">
   <si>
     <t>Long</t>
   </si>
@@ -136,7 +136,13 @@
     <t>Metrics by periods</t>
   </si>
   <si>
-    <t>Full metrics</t>
+    <t>Metrics for full period</t>
+  </si>
+  <si>
+    <t>Cumulative return</t>
+  </si>
+  <si>
+    <t>t-stat (mean)</t>
   </si>
 </sst>
 </file>
@@ -144,9 +150,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="165" formatCode="0.000%"/>
-    <numFmt numFmtId="168" formatCode="0.0000"/>
-    <numFmt numFmtId="171" formatCode="#,##0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.000%"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -225,14 +231,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -242,27 +245,25 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -615,7 +616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:O50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
@@ -635,82 +636,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="10" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="2" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4" t="s">
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4" t="s">
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4" t="s">
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="5" t="s">
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B3" s="7"/>
-      <c r="C3" s="7" t="s">
+      <c r="B3" s="6"/>
+      <c r="C3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="K3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="L3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="M3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="N3" s="7" t="s">
+      <c r="N3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="O3" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C4" s="1"/>
@@ -728,7 +729,7 @@
       <c r="O4" s="1"/>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C5" s="2">
@@ -749,13 +750,13 @@
       <c r="H5" s="2">
         <v>0.1204057165881969</v>
       </c>
-      <c r="I5" s="11">
+      <c r="I5" s="9">
         <v>0.64711161834743303</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="9">
         <v>-0.22251983912102541</v>
       </c>
-      <c r="K5" s="11">
+      <c r="K5" s="9">
         <v>1.6843150084627161</v>
       </c>
       <c r="L5" s="2">
@@ -772,7 +773,7 @@
       </c>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="2">
@@ -793,13 +794,13 @@
       <c r="H6" s="2">
         <v>9.8103110062493171E-2</v>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="9">
         <v>1.480686483156074</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="9">
         <v>1.4547155666209519</v>
       </c>
-      <c r="K6" s="11">
+      <c r="K6" s="9">
         <v>-0.45082522805195452</v>
       </c>
       <c r="L6" s="2">
@@ -816,7 +817,7 @@
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C7" s="2">
@@ -837,13 +838,13 @@
       <c r="H7" s="2">
         <v>7.3296008726515635E-2</v>
       </c>
-      <c r="I7" s="11">
+      <c r="I7" s="9">
         <v>3.590472162990733</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="9">
         <v>3.7342867131529589</v>
       </c>
-      <c r="K7" s="11">
+      <c r="K7" s="9">
         <v>-0.24022332785841019</v>
       </c>
       <c r="L7" s="2">
@@ -860,7 +861,7 @@
       </c>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="2">
@@ -881,13 +882,13 @@
       <c r="H8" s="2">
         <v>6.0619070340513677E-2</v>
       </c>
-      <c r="I8" s="11">
+      <c r="I8" s="9">
         <v>2.1901565102660179</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="9">
         <v>0.82150789710583383</v>
       </c>
-      <c r="K8" s="11">
+      <c r="K8" s="9">
         <v>1.7960483572059169</v>
       </c>
       <c r="L8" s="2">
@@ -904,7 +905,7 @@
       </c>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>25</v>
       </c>
       <c r="C9" s="2">
@@ -925,13 +926,13 @@
       <c r="H9" s="2">
         <v>7.5945237294059526E-2</v>
       </c>
-      <c r="I9" s="11">
+      <c r="I9" s="9">
         <v>-0.26085642578649387</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="9">
         <v>-6.7217022774122087E-2</v>
       </c>
-      <c r="K9" s="11">
+      <c r="K9" s="9">
         <v>-0.41474642876438178</v>
       </c>
       <c r="L9" s="2">
@@ -948,7 +949,7 @@
       </c>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C10" s="2">
@@ -969,13 +970,13 @@
       <c r="H10" s="2">
         <v>0.1037602926776751</v>
       </c>
-      <c r="I10" s="11">
+      <c r="I10" s="9">
         <v>1.150327004216692</v>
       </c>
-      <c r="J10" s="11">
+      <c r="J10" s="9">
         <v>0.83295491497180207</v>
       </c>
-      <c r="K10" s="11">
+      <c r="K10" s="9">
         <v>0.31728143354129851</v>
       </c>
       <c r="L10" s="2">
@@ -992,7 +993,7 @@
       </c>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>27</v>
       </c>
       <c r="C11" s="2">
@@ -1013,13 +1014,13 @@
       <c r="H11" s="2">
         <v>6.3292265797039463E-2</v>
       </c>
-      <c r="I11" s="11">
+      <c r="I11" s="9">
         <v>3.5219502081612259</v>
       </c>
-      <c r="J11" s="11">
+      <c r="J11" s="9">
         <v>1.9607987275290539</v>
       </c>
-      <c r="K11" s="11">
+      <c r="K11" s="9">
         <v>0.67112271172145621</v>
       </c>
       <c r="L11" s="2">
@@ -1036,7 +1037,7 @@
       </c>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C12" s="2">
@@ -1057,13 +1058,13 @@
       <c r="H12" s="2">
         <v>5.0252398724648151E-2</v>
       </c>
-      <c r="I12" s="11">
+      <c r="I12" s="9">
         <v>-0.59840559859905784</v>
       </c>
-      <c r="J12" s="11">
+      <c r="J12" s="9">
         <v>-0.90003542290500171</v>
       </c>
-      <c r="K12" s="11">
+      <c r="K12" s="9">
         <v>0.97835930137790339</v>
       </c>
       <c r="L12" s="2">
@@ -1080,7 +1081,7 @@
       </c>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>29</v>
       </c>
       <c r="C13" s="2">
@@ -1101,13 +1102,13 @@
       <c r="H13" s="2">
         <v>0.1160627861581847</v>
       </c>
-      <c r="I13" s="11">
+      <c r="I13" s="9">
         <v>1.178688404853657</v>
       </c>
-      <c r="J13" s="11">
+      <c r="J13" s="9">
         <v>1.596470767266239</v>
       </c>
-      <c r="K13" s="11">
+      <c r="K13" s="9">
         <v>-7.8488297431525217E-2</v>
       </c>
       <c r="L13" s="2">
@@ -1124,7 +1125,7 @@
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="5" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="2">
@@ -1145,13 +1146,13 @@
       <c r="H14" s="2">
         <v>0.12258051712162051</v>
       </c>
-      <c r="I14" s="11">
+      <c r="I14" s="9">
         <v>0.45493300968141892</v>
       </c>
-      <c r="J14" s="11">
+      <c r="J14" s="9">
         <v>0.70678354782001129</v>
       </c>
-      <c r="K14" s="11">
+      <c r="K14" s="9">
         <v>-0.70420809735321344</v>
       </c>
       <c r="L14" s="2">
@@ -1168,7 +1169,7 @@
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="5" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="2">
@@ -1189,13 +1190,13 @@
       <c r="H15" s="2">
         <v>0.19337436760144919</v>
       </c>
-      <c r="I15" s="11">
+      <c r="I15" s="9">
         <v>3.0136632759014041</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J15" s="9">
         <v>0.99152318871099898</v>
       </c>
-      <c r="K15" s="11">
+      <c r="K15" s="9">
         <v>0.58767348900790661</v>
       </c>
       <c r="L15" s="2">
@@ -1212,7 +1213,7 @@
       </c>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="5" t="s">
         <v>32</v>
       </c>
       <c r="C16" s="2">
@@ -1233,13 +1234,13 @@
       <c r="H16" s="2">
         <v>9.1375149737894304E-2</v>
       </c>
-      <c r="I16" s="11">
+      <c r="I16" s="9">
         <v>-0.48495805468663561</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="9">
         <v>-0.60897060668108327</v>
       </c>
-      <c r="K16" s="11">
+      <c r="K16" s="9">
         <v>0.15851972880123191</v>
       </c>
       <c r="L16" s="2">
@@ -1256,7 +1257,7 @@
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="5" t="s">
         <v>33</v>
       </c>
       <c r="C17" s="2">
@@ -1277,13 +1278,13 @@
       <c r="H17" s="2">
         <v>6.1792481791189117E-2</v>
       </c>
-      <c r="I17" s="11">
+      <c r="I17" s="9">
         <v>0.65901103337321787</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J17" s="9">
         <v>0.60005191657641233</v>
       </c>
-      <c r="K17" s="11">
+      <c r="K17" s="9">
         <v>0.12910777429226769</v>
       </c>
       <c r="L17" s="2">
@@ -1300,7 +1301,7 @@
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="5" t="s">
         <v>34</v>
       </c>
       <c r="C18" s="2">
@@ -1321,13 +1322,13 @@
       <c r="H18" s="2">
         <v>6.5684900838114957E-2</v>
       </c>
-      <c r="I18" s="11">
+      <c r="I18" s="9">
         <v>1.17682351278165</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18" s="9">
         <v>0.25080545538414262</v>
       </c>
-      <c r="K18" s="11">
+      <c r="K18" s="9">
         <v>2.002243176967704</v>
       </c>
       <c r="L18" s="2">
@@ -1344,7 +1345,7 @@
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C19" s="2">
@@ -1365,13 +1366,13 @@
       <c r="H19" s="2">
         <v>0.1014918934357685</v>
       </c>
-      <c r="I19" s="11">
+      <c r="I19" s="9">
         <v>0.64708622559015283</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19" s="9">
         <v>0.74608961942458052</v>
       </c>
-      <c r="K19" s="11">
+      <c r="K19" s="9">
         <v>0.10715273871539099</v>
       </c>
       <c r="L19" s="2">
@@ -1388,30 +1389,30 @@
       </c>
     </row>
     <row r="21" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="14"/>
-      <c r="B21" s="15" t="s">
+      <c r="A21" s="11"/>
+      <c r="B21" s="12" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="F22" s="10" t="s">
+      <c r="F22" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="13" t="s">
         <v>12</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -1428,7 +1429,7 @@
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="8"/>
+      <c r="B24" s="13"/>
       <c r="C24" s="1" t="s">
         <v>4</v>
       </c>
@@ -1443,22 +1444,22 @@
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="8"/>
+      <c r="B25" s="13"/>
       <c r="C25" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="7">
         <v>1.288265356544283</v>
       </c>
-      <c r="E25" s="9">
+      <c r="E25" s="7">
         <v>0.82067243276093194</v>
       </c>
-      <c r="F25" s="9">
+      <c r="F25" s="7">
         <v>0.47877693185360681</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B26" s="8"/>
+      <c r="B26" s="13"/>
       <c r="C26" s="1" t="s">
         <v>6</v>
       </c>
@@ -1473,7 +1474,7 @@
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="13" t="s">
         <v>13</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -1490,7 +1491,7 @@
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B28" s="8"/>
+      <c r="B28" s="13"/>
       <c r="C28" s="1" t="s">
         <v>4</v>
       </c>
@@ -1505,22 +1506,22 @@
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B29" s="8"/>
+      <c r="B29" s="13"/>
       <c r="C29" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D29" s="9">
+      <c r="D29" s="7">
         <v>0.40754715637292172</v>
       </c>
-      <c r="E29" s="9">
+      <c r="E29" s="7">
         <v>0.49898464198696058</v>
       </c>
-      <c r="F29" s="9">
+      <c r="F29" s="7">
         <v>-0.15411753974180989</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B30" s="8"/>
+      <c r="B30" s="13"/>
       <c r="C30" s="1" t="s">
         <v>6</v>
       </c>
@@ -1535,7 +1536,7 @@
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="13" t="s">
         <v>14</v>
       </c>
       <c r="C31" s="1" t="s">
@@ -1552,7 +1553,7 @@
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B32" s="8"/>
+      <c r="B32" s="13"/>
       <c r="C32" s="1" t="s">
         <v>4</v>
       </c>
@@ -1567,22 +1568,22 @@
       </c>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="8"/>
+      <c r="B33" s="13"/>
       <c r="C33" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D33" s="9">
+      <c r="D33" s="7">
         <v>0.40838161089665947</v>
       </c>
-      <c r="E33" s="9">
+      <c r="E33" s="7">
         <v>0.1246049235005454</v>
       </c>
-      <c r="F33" s="9">
+      <c r="F33" s="7">
         <v>0.43102272253820739</v>
       </c>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B34" s="8"/>
+      <c r="B34" s="13"/>
       <c r="C34" s="1" t="s">
         <v>6</v>
       </c>
@@ -1597,7 +1598,7 @@
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="13" t="s">
         <v>15</v>
       </c>
       <c r="C35" s="1" t="s">
@@ -1614,7 +1615,7 @@
       </c>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B36" s="8"/>
+      <c r="B36" s="13"/>
       <c r="C36" s="1" t="s">
         <v>4</v>
       </c>
@@ -1629,22 +1630,22 @@
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B37" s="8"/>
+      <c r="B37" s="13"/>
       <c r="C37" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D37" s="9">
+      <c r="D37" s="7">
         <v>0.78363627015788273</v>
       </c>
-      <c r="E37" s="9">
+      <c r="E37" s="7">
         <v>0.50043183056108875</v>
       </c>
-      <c r="F37" s="9">
+      <c r="F37" s="7">
         <v>0.64295602204972391</v>
       </c>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B38" s="8"/>
+      <c r="B38" s="13"/>
       <c r="C38" s="1" t="s">
         <v>6</v>
       </c>
@@ -1659,24 +1660,24 @@
       </c>
     </row>
     <row r="40" spans="2:6" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B40" s="16" t="s">
+      <c r="B40" s="12" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B41" s="10"/>
-      <c r="C41" s="10" t="s">
+      <c r="B41" s="8"/>
+      <c r="C41" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="D41" s="10" t="s">
+      <c r="D41" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="E41" s="10" t="s">
+      <c r="E41" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B42" s="12" t="s">
+      <c r="B42" s="15" t="s">
         <v>3</v>
       </c>
       <c r="C42" s="2">
@@ -1690,7 +1691,7 @@
       </c>
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B43" s="12" t="s">
+      <c r="B43" s="15" t="s">
         <v>4</v>
       </c>
       <c r="C43" s="2">
@@ -1704,85 +1705,113 @@
       </c>
     </row>
     <row r="44" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B44" s="12" t="s">
+      <c r="B44" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C44" s="11">
+      <c r="C44" s="9">
         <v>0.75040656880247902</v>
       </c>
-      <c r="D44" s="11">
+      <c r="D44" s="9">
         <v>0.55210077359813459</v>
       </c>
-      <c r="E44" s="11">
+      <c r="E44" s="9">
         <v>0.35779259572359717</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B45" s="12" t="s">
+      <c r="B45" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="C45" s="2">
+      <c r="C45" s="9">
         <v>-0.35294207802866429</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="9">
         <v>-0.32464832869616811</v>
       </c>
-      <c r="E45" s="2">
+      <c r="E45" s="9">
         <v>-0.237622952607738</v>
       </c>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B46" s="12" t="s">
+      <c r="B46" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="C46" s="9">
+        <v>7.0080035936562162</v>
+      </c>
+      <c r="D46" s="9">
+        <v>3.7132981944633858</v>
+      </c>
+      <c r="E46" s="9">
+        <v>0.5733554136079444</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B47" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C47" s="9">
+        <v>3.2065610882211741</v>
+      </c>
+      <c r="D47" s="9">
+        <v>2.430814822421508</v>
+      </c>
+      <c r="E47" s="9">
+        <v>1.3857247646338151</v>
+      </c>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B48" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="2">
+      <c r="C48" s="2">
         <v>0.66111111111111109</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D48" s="2">
         <v>0.6</v>
       </c>
-      <c r="E46" s="2">
+      <c r="E48" s="2">
         <v>0.52777777777777779</v>
       </c>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B47" s="12" t="s">
+    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B49" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C47" s="2">
+      <c r="C49" s="2">
         <v>0.2063805651783254</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D49" s="2">
         <v>0.22826799032119929</v>
       </c>
-      <c r="E47" s="2">
+      <c r="E49" s="2">
         <v>9.4944563566654525E-2</v>
       </c>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B48" s="12" t="s">
+    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B50" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="C48" s="2">
+      <c r="C50" s="2">
         <v>-0.26507709364416349</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D50" s="2">
         <v>-0.22012739418385879</v>
       </c>
-      <c r="E48" s="2">
+      <c r="E50" s="2">
         <v>-0.13793125191391131</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="B23:B26"/>
     <mergeCell ref="B27:B30"/>
     <mergeCell ref="B31:B34"/>
     <mergeCell ref="B35:B38"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:H2"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="B23:B26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>